<commit_message>
feat: test-data-gen 도구 추가
</commit_message>
<xml_diff>
--- a/02.tools/02.excel-reporter/결과/report_2026-06-17.xlsx
+++ b/02.tools/02.excel-reporter/결과/report_2026-06-17.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="전체 버그 목록" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="담당자별 현황" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="심각도별 통계" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="요약 대시보드" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="발견자별 현황" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="플랫폼별 현황" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="심각도·우선순위" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="요약 대시보드" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,6 +35,9 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="004472C4"/>
       <sz val="16"/>
     </font>
@@ -43,7 +47,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -62,12 +66,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FF6600"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFC000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="0070AD47"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BFBFBF"/>
       </patternFill>
     </fill>
   </fills>
@@ -83,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -91,22 +105,32 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -181,193 +205,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>담당자별 버그 현황</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'담당자별 현황'!B1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'담당자별 현황'!$A$2:$A$4</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'담당자별 현황'!$B$2:$B$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'담당자별 현황'!C1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'담당자별 현황'!$A$2:$A$4</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'담당자별 현황'!$C$2:$C$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="2"/>
-          <order val="2"/>
-          <tx>
-            <strRef>
-              <f>'담당자별 현황'!D1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'담당자별 현황'!$A$2:$A$4</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'담당자별 현황'!$D$2:$D$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>담당자</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>건수</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>1</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="5400000" cy="2700000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -659,16 +496,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -689,22 +530,42 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>담당자</t>
+          <t>우선순위</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>플랫폼</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>버전</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>상태</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>발견자</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>발견일</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>해결일</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>재현율</t>
         </is>
       </c>
     </row>
@@ -726,22 +587,42 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>v1.2.34</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
           <t>홍길동</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>해결</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>2026-06-10</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
         </is>
       </c>
     </row>
@@ -758,26 +639,44 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>v1.2.34</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
           <t>이철수</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>진행중</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>2026-06-11</t>
         </is>
       </c>
-      <c r="G3" s="3" t="n">
-        <v/>
+      <c r="J3" s="3" t="inlineStr"/>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>8/10</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -793,27 +692,47 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>v1.2.33</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
           <t>홍길동</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>해결</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>2026-06-11</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>5/10</t>
         </is>
       </c>
     </row>
@@ -835,57 +754,95 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>iOS</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>v1.2.34</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
           <t>박영희</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>2026-06-12</t>
         </is>
       </c>
-      <c r="G5" s="2" t="n">
-        <v/>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>BUG-005</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>UI 텍스트 겹침</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>v1.2.33</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>이철수</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>해결</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>2026-06-12</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>3/10</t>
         </is>
       </c>
     </row>
@@ -902,27 +859,41 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>v1.2.34</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
           <t>박영희</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>진행중</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="G7" s="3" t="n">
-        <v/>
-      </c>
+      <c r="J7" s="3" t="inlineStr"/>
+      <c r="K7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -937,26 +908,44 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>v1.2.34</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
           <t>홍길동</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="G8" s="3" t="n">
-        <v/>
+      <c r="J8" s="3" t="inlineStr"/>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>6/10</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -977,22 +966,42 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>iOS</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>v1.2.34</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
           <t>이철수</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>해결</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>9/10</t>
         </is>
       </c>
     </row>
@@ -1007,19 +1016,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>담당자</t>
+          <t>발견자</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -1037,58 +1047,71 @@
           <t>해결</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>합계</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>박영희</t>
         </is>
       </c>
-      <c r="B2" s="5" t="n">
+      <c r="B2" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="5" t="n">
+      <c r="C2" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="D2" s="9" t="n">
         <v>0</v>
       </c>
+      <c r="E2" s="1" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>이철수</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n">
+      <c r="B3" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C3" s="5" t="n">
+      <c r="C3" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="D3" s="9" t="n">
         <v>2</v>
       </c>
+      <c r="E3" s="1" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>홍길동</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B4" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="C4" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D4" s="9" t="n">
         <v>2</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1098,52 +1121,112 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>심각도</t>
+          <t>플랫폼</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>건수</t>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>합계</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="n">
-        <v>3</v>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="11" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>Major</t>
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>PC</t>
         </is>
       </c>
       <c r="B3" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="C3" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="11" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="B4" s="8" t="n">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>iOS</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="11" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1158,15 +1241,131 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>심각도</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>건수</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>우선순위</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>건수</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>📊 QA 버그 리포트 요약</t>
         </is>
@@ -1177,12 +1376,12 @@
       <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>수치</t>
         </is>
@@ -1201,88 +1400,206 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>해결률</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>상태별</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>건수</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
           <t>해결</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B8" s="9" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>진행중</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B9" s="8" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>미해결</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B10" s="7" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>해결률</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>50.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-      <c r="B9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>심각도별</t>
         </is>
       </c>
-      <c r="B10" s="1" t="inlineStr">
+      <c r="B12" s="1" t="inlineStr">
         <is>
           <t>건수</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B13" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>우선순위별</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t>건수</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>플랫폼별</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
+        <is>
+          <t>건수</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>iOS</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>